<commit_message>
3d layout display changes
</commit_message>
<xml_diff>
--- a/data/om_loading_master.xlsx
+++ b/data/om_loading_master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rishitgupta/Documents/Test/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89280B6-B475-4D49-84C5-25B46FF23D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC306874-7D72-7146-A4E6-E40790592A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="155">
   <si>
     <t>Truck_ID</t>
   </si>
@@ -497,6 +497,12 @@
   </si>
   <si>
     <t>Must_Upright</t>
+  </si>
+  <si>
+    <t>DKT-1016</t>
+  </si>
+  <si>
+    <t>Bulbs</t>
   </si>
 </sst>
 </file>
@@ -908,7 +914,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DocketMasterTable" displayName="DocketMasterTable" ref="A1:N16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DocketMasterTable" displayName="DocketMasterTable" ref="A1:N17">
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Docket_No"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Destination"/>
@@ -1344,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
@@ -1440,11 +1446,11 @@
         <v>43</v>
       </c>
       <c r="L2" s="6">
-        <f t="shared" ref="L2:L16" si="0">G2*H2</f>
+        <f t="shared" ref="L2:L17" si="0">G2*H2</f>
         <v>336</v>
       </c>
       <c r="M2" s="6">
-        <f t="shared" ref="M2:M16" si="1">D2*E2*F2*H2</f>
+        <f t="shared" ref="M2:M17" si="1">D2*E2*F2*H2</f>
         <v>50.399999999999991</v>
       </c>
       <c r="N2" s="3" t="s">
@@ -2093,6 +2099,52 @@
       </c>
       <c r="N16" s="3" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17">
+        <v>1.5</v>
+      </c>
+      <c r="E17">
+        <v>2.8</v>
+      </c>
+      <c r="F17">
+        <v>0.8</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>550</v>
+      </c>
+      <c r="I17" t="s">
+        <v>42</v>
+      </c>
+      <c r="J17" t="s">
+        <v>43</v>
+      </c>
+      <c r="K17" t="s">
+        <v>43</v>
+      </c>
+      <c r="L17" s="6">
+        <f t="shared" si="0"/>
+        <v>1650</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="1"/>
+        <v>1847.9999999999998</v>
+      </c>
+      <c r="N17" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>